<commit_message>
Follow NNR's monitoring sheet: HBL format, arrastre cut-off, sheet import
- HBL No. is NNRMNL{POD}{F|L}{seq}, one running number starting after
  HBL_START_AFTER; destination code from a city dictionary or UN/LOCODE.
- Arrastre deadline is the entered arrastre cut-off; new fields for
  declaration c/o and broker, docs sent to carrier, PART OF link.
- Board, raw Excel sheet and import share the sheet's 24 columns and
  3-row header; HBL is the main reference.
- Importer reads the sheet as is (xlsx or csv): year inference, history
  cut-off, shipper typo merging, DIRECT BL, PART OF, rows-to-fix file.
- Monthly on-time metrics exclude imported history.
- Each test file starts from an empty database (order-independent).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M4G4D3xFxHWM88UFn3zYuP
</commit_message>
<xml_diff>
--- a/docs/import-template.xlsx
+++ b/docs/import-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="49">
   <si>
     <t>Job No.</t>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t>Pre-advise Sent</t>
+  </si>
+  <si>
+    <t>Arrastre Cut-off</t>
   </si>
   <si>
     <t>Export Declaration</t>
@@ -535,13 +538,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AA3"/>
+  <dimension ref="A1:AB3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="27" width="20" customWidth="1"/>
+    <col min="1" max="28" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -623,171 +626,180 @@
       <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="O2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R2" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="S2" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="T2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="U2" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="V2" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="W2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="X2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Y2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Z2" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="AA2" t="s">
-        <v>27</v>
+        <v>40</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="M3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="O3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P3" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="Q3" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="R3" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="S3" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="T3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="U3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="V3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="W3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="X3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Y3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Z3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AA3" t="s">
-        <v>47</v>
+        <v>28</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>